<commit_message>
Added the storage deal and BRRRR sheets. Hooked up the new palettes and formatting.
</commit_message>
<xml_diff>
--- a/sheets/freelance-and-side-hustle/freelance-pnl-tracker/freelance-pnl-tracker.xlsx
+++ b/sheets/freelance-and-side-hustle/freelance-pnl-tracker/freelance-pnl-tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\My Drive\000_drive_drive\600_PROJECTS\modelstack\sheets\freelance-and-side-hustle\freelance-pnl-tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6538987-62E0-4A30-ABAD-78487F6EFB1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BA5791B-30D2-4981-868A-6416D9BC0756}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue Log" sheetId="1" r:id="rId1"/>
@@ -1006,7 +1006,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1027,6 +1027,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="1" tint="0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1052,7 +1058,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1105,6 +1111,9 @@
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1198,8 +1207,8 @@
       <xdr:row>5</xdr:row>
       <xdr:rowOff>133680</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="5" name="Ink 4">
@@ -1218,7 +1227,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="5" name="Ink 4">
@@ -3633,7 +3642,7 @@
         <v>114</v>
       </c>
       <c r="F34" s="16" t="str">
-        <f t="shared" ref="F34:F65" si="3">IF(E34="Meals (50%)","Partial",IF(E34="Other","Check","Yes"))</f>
+        <f t="shared" ref="F34:F50" si="3">IF(E34="Meals (50%)","Partial",IF(E34="Other","Check","Yes"))</f>
         <v>Yes</v>
       </c>
       <c r="G34" s="15">
@@ -4787,34 +4796,34 @@
       </c>
     </row>
     <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="15">
+      <c r="B14" s="31">
         <f t="shared" ref="B14:G14" si="6">SUM(B2:B13)</f>
         <v>56980</v>
       </c>
-      <c r="C14" s="15">
+      <c r="C14" s="31">
         <f t="shared" si="6"/>
         <v>1293</v>
       </c>
-      <c r="D14" s="15">
+      <c r="D14" s="31">
         <f t="shared" si="6"/>
         <v>55687</v>
       </c>
-      <c r="E14" s="15">
+      <c r="E14" s="31">
         <f t="shared" si="6"/>
         <v>4641.4599999999991</v>
       </c>
-      <c r="F14" s="15">
+      <c r="F14" s="31">
         <f t="shared" si="6"/>
         <v>4745.8599999999997</v>
       </c>
-      <c r="G14" s="15">
+      <c r="G14" s="31">
         <f t="shared" si="6"/>
         <v>51045.54</v>
       </c>
-      <c r="H14" s="17">
+      <c r="H14" s="32">
         <f t="shared" si="2"/>
         <v>0.89585012285012289</v>
       </c>

</xml_diff>